<commit_message>
Restore missing evaluation artifacts after project refactor
</commit_message>
<xml_diff>
--- a/data/features/selected_features.xlsx
+++ b/data/features/selected_features.xlsx
@@ -521,7 +521,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>19-07-2026 07:45:32</t>
+          <t>19-07-2026 09:04:58</t>
         </is>
       </c>
     </row>
@@ -1554,7 +1554,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>19-07-2026 07:45:32</t>
+          <t>19-07-2026 09:04:58</t>
         </is>
       </c>
     </row>

</xml_diff>